<commit_message>
perf(buyer): implement batch pre-fetching to eliminate N+1 queries in PO child endpoints perf(buyer): optimize remaining slow endpoints by reducing query counts and improving performance
</commit_message>
<xml_diff>
--- a/MSQ App Version History.xlsx
+++ b/MSQ App Version History.xlsx
@@ -14,6 +14,8 @@
     <sheet name="v1.0.1.2 Changelog" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Version History Summary" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="Deployment Notes" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="v1.0.3.0 Changelog" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="v1.0.3.1 Changelog" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191028" fullCalcOnLoad="1"/>
@@ -25,7 +27,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="16">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -72,8 +74,46 @@
       <color rgb="00FFFFFF"/>
       <sz val="12"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="000070C0"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FF0000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FF8C00"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="007030A0"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="0070AD47"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00808080"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -104,8 +144,23 @@
         <bgColor rgb="00E74C3C"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F3864"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -113,11 +168,39 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00CCCCCC"/>
+      </left>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00DDDDDD"/>
+      </left>
+      <right style="thin">
+        <color rgb="00DDDDDD"/>
+      </right>
+      <top style="thin">
+        <color rgb="00DDDDDD"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00DDDDDD"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -173,6 +256,54 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -541,7 +672,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9.7109375" customWidth="1" style="3" min="1" max="1"/>
@@ -585,168 +716,168 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="24" t="inlineStr">
+        <is>
+          <t>1.0.3.1</t>
+        </is>
+      </c>
+      <c r="B2" s="24" t="inlineStr">
+        <is>
+          <t>2026-02-24</t>
+        </is>
+      </c>
+      <c r="C2" s="24" t="inlineStr">
+        <is>
+          <t>Released</t>
+        </is>
+      </c>
+      <c r="D2" s="24" t="inlineStr">
+        <is>
+          <t>Production</t>
+        </is>
+      </c>
+      <c r="E2" s="24" t="inlineStr">
+        <is>
+          <t>DevOps Team</t>
+        </is>
+      </c>
+      <c r="F2" s="24" t="inlineStr">
+        <is>
+          <t>Latest - 42 features/fixes</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="24" t="inlineStr">
+        <is>
+          <t>1.0.3.0</t>
+        </is>
+      </c>
+      <c r="B3" s="24" t="inlineStr">
+        <is>
+          <t>2026-02-07</t>
+        </is>
+      </c>
+      <c r="C3" s="24" t="inlineStr">
+        <is>
+          <t>Released</t>
+        </is>
+      </c>
+      <c r="D3" s="24" t="inlineStr">
+        <is>
+          <t>Production</t>
+        </is>
+      </c>
+      <c r="E3" s="24" t="inlineStr">
+        <is>
+          <t>DevOps Team</t>
+        </is>
+      </c>
+      <c r="F3" s="24" t="inlineStr">
+        <is>
+          <t>Previous - 47 features/fixes</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
         <is>
           <t>1.0.2.1</t>
         </is>
       </c>
-      <c r="B2" s="22" t="n">
+      <c r="B4" s="22" t="n">
         <v>46040</v>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>Released</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>Production</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>DevOps Team</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Latest - 68 features/fixes</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Previous - 68 features/fixes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>1.0.1.5</t>
         </is>
       </c>
-      <c r="B3" s="5" t="n">
+      <c r="B5" s="5" t="n">
         <v>46022</v>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>Released</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>Production</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>DevOps Team</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="F5" s="4" t="inlineStr">
         <is>
           <t>Previous - 22 features/fixes</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
         <is>
           <t>1.0.1.4</t>
         </is>
       </c>
-      <c r="B4" s="2" t="n">
+      <c r="B6" s="2" t="n">
         <v>46011</v>
       </c>
-      <c r="C4" s="1" t="inlineStr">
+      <c r="C6" s="1" t="inlineStr">
         <is>
           <t>Released</t>
         </is>
       </c>
-      <c r="D4" s="1" t="inlineStr">
+      <c r="D6" s="1" t="inlineStr">
         <is>
           <t>Production</t>
         </is>
       </c>
-      <c r="E4" s="1" t="inlineStr">
+      <c r="E6" s="1" t="inlineStr">
         <is>
           <t>DevOps Team</t>
         </is>
       </c>
-      <c r="F4" s="1" t="inlineStr">
+      <c r="F6" s="1" t="inlineStr">
         <is>
           <t>Latest - 20 features/fixes</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>1.0.1.3</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>2025-12-16</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>Released</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>Production</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>DevOps Team</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>Latest - 15 features/fixes</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>1.0.1.2</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>2025-12-12</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>Released</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>Production</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>DevOps Team</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>Stable - 35 features/fixes</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>1.0.1.1</t>
+          <t>1.0.1.3</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>2025-10-12</t>
+          <t>2025-12-16</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -766,37 +897,101 @@
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>Previous - 15 bug fixes</t>
+          <t>Latest - 15 features/fixes</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
+          <t>1.0.1.2</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>2025-12-12</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Released</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Production</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>DevOps Team</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>Stable - 35 features/fixes</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>1.0.1.1</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>2025-10-12</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Released</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Production</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>DevOps Team</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>Previous - 15 bug fixes</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
           <t>1.0.1.0</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>2025-10-01</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
         <is>
           <t>Archived</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="D10" s="3" t="inlineStr">
         <is>
           <t>Production</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="E10" s="3" t="inlineStr">
         <is>
           <t>DevOps Team</t>
         </is>
       </c>
-      <c r="F8" s="3" t="inlineStr">
+      <c r="F10" s="3" t="inlineStr">
         <is>
           <t>Legacy version</t>
         </is>
@@ -804,6 +999,1536 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G43"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="65" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="25" t="inlineStr">
+        <is>
+          <t>Item#</t>
+        </is>
+      </c>
+      <c r="B1" s="25" t="inlineStr">
+        <is>
+          <t>Release Date</t>
+        </is>
+      </c>
+      <c r="C1" s="25" t="inlineStr">
+        <is>
+          <t>Component</t>
+        </is>
+      </c>
+      <c r="D1" s="25" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="E1" s="25" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="F1" s="25" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="G1" s="25" t="inlineStr">
+        <is>
+          <t>Severity</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="26" t="inlineStr">
+        <is>
+          <t>2026-02-08</t>
+        </is>
+      </c>
+      <c r="C2" s="26" t="inlineStr">
+        <is>
+          <t>Buyer</t>
+        </is>
+      </c>
+      <c r="D2" s="27" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E2" s="26" t="inlineStr">
+        <is>
+          <t>Buyer raw material list implemented for material management</t>
+        </is>
+      </c>
+      <c r="F2" s="26" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G2" s="32" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="18" customHeight="1">
+      <c r="A3" s="29" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="29" t="inlineStr">
+        <is>
+          <t>2026-02-09</t>
+        </is>
+      </c>
+      <c r="C3" s="29" t="inlineStr">
+        <is>
+          <t>Global Search</t>
+        </is>
+      </c>
+      <c r="D3" s="30" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E3" s="29" t="inlineStr">
+        <is>
+          <t>Global autocomplete search for materials and labours with debouncing and race condition handling</t>
+        </is>
+      </c>
+      <c r="F3" s="29" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G3" s="31" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="18" customHeight="1">
+      <c r="A4" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="26" t="inlineStr">
+        <is>
+          <t>2026-02-09</t>
+        </is>
+      </c>
+      <c r="C4" s="26" t="inlineStr">
+        <is>
+          <t>Catalog Management</t>
+        </is>
+      </c>
+      <c r="D4" s="27" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E4" s="26" t="inlineStr">
+        <is>
+          <t>Catalog items management routes and UI components: CatalogItemsManager, AddCatalogItemModal, CatalogImportModal</t>
+        </is>
+      </c>
+      <c r="F4" s="26" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G4" s="28" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" s="29" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="29" t="inlineStr">
+        <is>
+          <t>2026-02-09</t>
+        </is>
+      </c>
+      <c r="C5" s="29" t="inlineStr">
+        <is>
+          <t>BOQ Day Extension</t>
+        </is>
+      </c>
+      <c r="D5" s="30" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E5" s="29" t="inlineStr">
+        <is>
+          <t>Day extension status in BOQ assignments with blinking alert animation for pending requests</t>
+        </is>
+      </c>
+      <c r="F5" s="29" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G5" s="33" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="18" customHeight="1">
+      <c r="A6" s="26" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="26" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="C6" s="26" t="inlineStr">
+        <is>
+          <t>IMR Approval</t>
+        </is>
+      </c>
+      <c r="D6" s="27" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E6" s="26" t="inlineStr">
+        <is>
+          <t>New route to send all materials directly to M2 Store without POChild; enhanced internal request approval logging</t>
+        </is>
+      </c>
+      <c r="F6" s="26" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G6" s="28" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="18" customHeight="1">
+      <c r="A7" s="29" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="29" t="inlineStr">
+        <is>
+          <t>2026-02-19</t>
+        </is>
+      </c>
+      <c r="C7" s="29" t="inlineStr">
+        <is>
+          <t>Vendor Inspection</t>
+        </is>
+      </c>
+      <c r="D7" s="30" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E7" s="29" t="inlineStr">
+        <is>
+          <t>Vendor inspection service with endpoints for managing inspections and vendor return requests</t>
+        </is>
+      </c>
+      <c r="F7" s="29" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G7" s="31" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="18" customHeight="1">
+      <c r="A8" s="26" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="26" t="inlineStr">
+        <is>
+          <t>2026-02-19</t>
+        </is>
+      </c>
+      <c r="C8" s="26" t="inlineStr">
+        <is>
+          <t>Return Edit</t>
+        </is>
+      </c>
+      <c r="D8" s="27" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E8" s="26" t="inlineStr">
+        <is>
+          <t>Edit and resubmit functionality for TD-rejected return requests</t>
+        </is>
+      </c>
+      <c r="F8" s="26" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G8" s="28" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="A9" s="29" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="29" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="C9" s="29" t="inlineStr">
+        <is>
+          <t>Email Notifications</t>
+        </is>
+      </c>
+      <c r="D9" s="30" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E9" s="29" t="inlineStr">
+        <is>
+          <t>BOQ and purchase email notifications for stakeholders</t>
+        </is>
+      </c>
+      <c r="F9" s="29" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G9" s="31" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="A10" s="26" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="26" t="inlineStr">
+        <is>
+          <t>2026-02-23</t>
+        </is>
+      </c>
+      <c r="C10" s="26" t="inlineStr">
+        <is>
+          <t>LPO PDF Storage</t>
+        </is>
+      </c>
+      <c r="D10" s="27" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E10" s="26" t="inlineStr">
+        <is>
+          <t>LPO PDF URL column added to change_requests and po_child tables; LPO PDF generation and Supabase storage upload</t>
+        </is>
+      </c>
+      <c r="F10" s="26" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G10" s="28" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="A11" s="29" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="29" t="inlineStr">
+        <is>
+          <t>2026-02-23</t>
+        </is>
+      </c>
+      <c r="C11" s="29" t="inlineStr">
+        <is>
+          <t>CC Email Management</t>
+        </is>
+      </c>
+      <c r="D11" s="30" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E11" s="29" t="inlineStr">
+        <is>
+          <t>Dynamic CC email management with admin and buyer configuration for outgoing emails</t>
+        </is>
+      </c>
+      <c r="F11" s="29" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G11" s="31" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="A12" s="26" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="26" t="inlineStr">
+        <is>
+          <t>2026-02-23</t>
+        </is>
+      </c>
+      <c r="C12" s="26" t="inlineStr">
+        <is>
+          <t>Vendor Return Image</t>
+        </is>
+      </c>
+      <c r="D12" s="27" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E12" s="26" t="inlineStr">
+        <is>
+          <t>All roles can view images in vendor return material flow</t>
+        </is>
+      </c>
+      <c r="F12" s="26" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G12" s="32" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="18" customHeight="1">
+      <c r="A13" s="29" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="29" t="inlineStr">
+        <is>
+          <t>2026-02-23</t>
+        </is>
+      </c>
+      <c r="C13" s="29" t="inlineStr">
+        <is>
+          <t>Email Templates</t>
+        </is>
+      </c>
+      <c r="D13" s="30" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E13" s="29" t="inlineStr">
+        <is>
+          <t>Enhanced email templates with file upload capabilities across various components</t>
+        </is>
+      </c>
+      <c r="F13" s="29" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G13" s="33" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="18" customHeight="1">
+      <c r="A14" s="26" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="26" t="inlineStr">
+        <is>
+          <t>2026-02-23</t>
+        </is>
+      </c>
+      <c r="C14" s="26" t="inlineStr">
+        <is>
+          <t>Vendor Return Flow</t>
+        </is>
+      </c>
+      <c r="D14" s="27" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E14" s="26" t="inlineStr">
+        <is>
+          <t>New vendor selection flow for vendor return material processing</t>
+        </is>
+      </c>
+      <c r="F14" s="26" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G14" s="28" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="18" customHeight="1">
+      <c r="A15" s="29" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="29" t="inlineStr">
+        <is>
+          <t>2026-02-09</t>
+        </is>
+      </c>
+      <c r="C15" s="29" t="inlineStr">
+        <is>
+          <t>BOQ/Catalog</t>
+        </is>
+      </c>
+      <c r="D15" s="35" t="inlineStr">
+        <is>
+          <t>Enhancement</t>
+        </is>
+      </c>
+      <c r="E15" s="29" t="inlineStr">
+        <is>
+          <t>Master item search functionality improvements and UI updates for suggestions and existing item handling</t>
+        </is>
+      </c>
+      <c r="F15" s="29" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G15" s="33" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="18" customHeight="1">
+      <c r="A16" s="26" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="26" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="C16" s="26" t="inlineStr">
+        <is>
+          <t>Rate Limiting</t>
+        </is>
+      </c>
+      <c r="D16" s="34" t="inlineStr">
+        <is>
+          <t>Enhancement</t>
+        </is>
+      </c>
+      <c r="E16" s="26" t="inlineStr">
+        <is>
+          <t>Server port updated to 5001 and API rate limits increased to accommodate polling and multiple concurrent users</t>
+        </is>
+      </c>
+      <c r="F16" s="26" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G16" s="28" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="18" customHeight="1">
+      <c r="A17" s="29" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="29" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="C17" s="29" t="inlineStr">
+        <is>
+          <t>Estimator Roles</t>
+        </is>
+      </c>
+      <c r="D17" s="35" t="inlineStr">
+        <is>
+          <t>Enhancement</t>
+        </is>
+      </c>
+      <c r="E17" s="29" t="inlineStr">
+        <is>
+          <t>New role checks for estimators in permission functions and enhanced material processing with size and sub-item name</t>
+        </is>
+      </c>
+      <c r="F17" s="29" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G17" s="33" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="18" customHeight="1">
+      <c r="A18" s="26" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="26" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="C18" s="26" t="inlineStr">
+        <is>
+          <t>BOQ Sub-items PDF</t>
+        </is>
+      </c>
+      <c r="D18" s="34" t="inlineStr">
+        <is>
+          <t>Enhancement</t>
+        </is>
+      </c>
+      <c r="E18" s="26" t="inlineStr">
+        <is>
+          <t>Added description, brand, and size fields to sub-items in internal Excel and client PDF generation</t>
+        </is>
+      </c>
+      <c r="F18" s="26" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G18" s="32" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="18" customHeight="1">
+      <c r="A19" s="29" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="29" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="C19" s="29" t="inlineStr">
+        <is>
+          <t>Purchase Orders UI</t>
+        </is>
+      </c>
+      <c r="D19" s="35" t="inlineStr">
+        <is>
+          <t>Enhancement</t>
+        </is>
+      </c>
+      <c r="E19" s="29" t="inlineStr">
+        <is>
+          <t>Refactored PurchaseOrders page with improved sorting and display for completed and rejected statuses</t>
+        </is>
+      </c>
+      <c r="F19" s="29" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G19" s="33" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="18" customHeight="1">
+      <c r="A20" s="26" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="26" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="C20" s="26" t="inlineStr">
+        <is>
+          <t>Project Navigation</t>
+        </is>
+      </c>
+      <c r="D20" s="34" t="inlineStr">
+        <is>
+          <t>Enhancement</t>
+        </is>
+      </c>
+      <c r="E20" s="26" t="inlineStr">
+        <is>
+          <t>Enhanced project navigation logic based on user roles</t>
+        </is>
+      </c>
+      <c r="F20" s="26" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G20" s="37" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="18" customHeight="1">
+      <c r="A21" s="29" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="29" t="inlineStr">
+        <is>
+          <t>2026-02-13</t>
+        </is>
+      </c>
+      <c r="C21" s="29" t="inlineStr">
+        <is>
+          <t>Internal Revisions</t>
+        </is>
+      </c>
+      <c r="D21" s="35" t="inlineStr">
+        <is>
+          <t>Enhancement</t>
+        </is>
+      </c>
+      <c r="E21" s="29" t="inlineStr">
+        <is>
+          <t>Internal revisions API enhanced with caching and performance improvements</t>
+        </is>
+      </c>
+      <c r="F21" s="29" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G21" s="33" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="18" customHeight="1">
+      <c r="A22" s="26" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="26" t="inlineStr">
+        <is>
+          <t>2026-02-18</t>
+        </is>
+      </c>
+      <c r="C22" s="26" t="inlineStr">
+        <is>
+          <t>Vendor Status</t>
+        </is>
+      </c>
+      <c r="D22" s="34" t="inlineStr">
+        <is>
+          <t>Enhancement</t>
+        </is>
+      </c>
+      <c r="E22" s="26" t="inlineStr">
+        <is>
+          <t>Vendor approval status displayed in estimator and PM roles</t>
+        </is>
+      </c>
+      <c r="F22" s="26" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G22" s="32" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="18" customHeight="1">
+      <c r="A23" s="29" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="29" t="inlineStr">
+        <is>
+          <t>2026-02-19</t>
+        </is>
+      </c>
+      <c r="C23" s="29" t="inlineStr">
+        <is>
+          <t>Online/Offline Status</t>
+        </is>
+      </c>
+      <c r="D23" s="35" t="inlineStr">
+        <is>
+          <t>Enhancement</t>
+        </is>
+      </c>
+      <c r="E23" s="29" t="inlineStr">
+        <is>
+          <t>Automatic online/offline status detection and tracking</t>
+        </is>
+      </c>
+      <c r="F23" s="29" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G23" s="33" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="18" customHeight="1">
+      <c r="A24" s="26" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="26" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="C24" s="26" t="inlineStr">
+        <is>
+          <t>Buyer Material</t>
+        </is>
+      </c>
+      <c r="D24" s="34" t="inlineStr">
+        <is>
+          <t>Enhancement</t>
+        </is>
+      </c>
+      <c r="E24" s="26" t="inlineStr">
+        <is>
+          <t>Buyer material transfer shows PM name for better tracking</t>
+        </is>
+      </c>
+      <c r="F24" s="26" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G24" s="37" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="18" customHeight="1">
+      <c r="A25" s="29" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="29" t="inlineStr">
+        <is>
+          <t>2026-02-23</t>
+        </is>
+      </c>
+      <c r="C25" s="29" t="inlineStr">
+        <is>
+          <t>CR/TD Enhancement</t>
+        </is>
+      </c>
+      <c r="D25" s="35" t="inlineStr">
+        <is>
+          <t>Enhancement</t>
+        </is>
+      </c>
+      <c r="E25" s="29" t="inlineStr">
+        <is>
+          <t>Change request and TD controllers enhanced with vendor details and performance improvements</t>
+        </is>
+      </c>
+      <c r="F25" s="29" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G25" s="31" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="18" customHeight="1">
+      <c r="A26" s="26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="26" t="inlineStr">
+        <is>
+          <t>2026-02-23</t>
+        </is>
+      </c>
+      <c r="C26" s="26" t="inlineStr">
+        <is>
+          <t>Code Refactor</t>
+        </is>
+      </c>
+      <c r="D26" s="34" t="inlineStr">
+        <is>
+          <t>Enhancement</t>
+        </is>
+      </c>
+      <c r="E26" s="26" t="inlineStr">
+        <is>
+          <t>Code structure refactored across multiple components for improved readability and maintainability</t>
+        </is>
+      </c>
+      <c r="F26" s="26" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G26" s="37" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="18" customHeight="1">
+      <c r="A27" s="29" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="29" t="inlineStr">
+        <is>
+          <t>2026-02-09</t>
+        </is>
+      </c>
+      <c r="C27" s="29" t="inlineStr">
+        <is>
+          <t>Material Entry</t>
+        </is>
+      </c>
+      <c r="D27" s="31" t="inlineStr">
+        <is>
+          <t>Fix</t>
+        </is>
+      </c>
+      <c r="E27" s="29" t="inlineStr">
+        <is>
+          <t>Material, item, and sub-item entry fixes</t>
+        </is>
+      </c>
+      <c r="F27" s="29" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G27" s="33" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="18" customHeight="1">
+      <c r="A28" s="26" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="26" t="inlineStr">
+        <is>
+          <t>2026-02-09</t>
+        </is>
+      </c>
+      <c r="C28" s="26" t="inlineStr">
+        <is>
+          <t>Buyer Sub-item</t>
+        </is>
+      </c>
+      <c r="D28" s="28" t="inlineStr">
+        <is>
+          <t>Fix</t>
+        </is>
+      </c>
+      <c r="E28" s="26" t="inlineStr">
+        <is>
+          <t>Buyer sub-item display and processing fixed</t>
+        </is>
+      </c>
+      <c r="F28" s="26" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G28" s="32" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="18" customHeight="1">
+      <c r="A29" s="29" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="29" t="inlineStr">
+        <is>
+          <t>2026-02-09</t>
+        </is>
+      </c>
+      <c r="C29" s="29" t="inlineStr">
+        <is>
+          <t>Estimator Budget</t>
+        </is>
+      </c>
+      <c r="D29" s="31" t="inlineStr">
+        <is>
+          <t>Fix</t>
+        </is>
+      </c>
+      <c r="E29" s="29" t="inlineStr">
+        <is>
+          <t>Estimator budget calculation fix</t>
+        </is>
+      </c>
+      <c r="F29" s="29" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G29" s="33" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="18" customHeight="1">
+      <c r="A30" s="26" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="26" t="inlineStr">
+        <is>
+          <t>2026-02-09</t>
+        </is>
+      </c>
+      <c r="C30" s="26" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="D30" s="28" t="inlineStr">
+        <is>
+          <t>Fix</t>
+        </is>
+      </c>
+      <c r="E30" s="26" t="inlineStr">
+        <is>
+          <t>Build configuration fix</t>
+        </is>
+      </c>
+      <c r="F30" s="26" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G30" s="37" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="18" customHeight="1">
+      <c r="A31" s="29" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="29" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="C31" s="29" t="inlineStr">
+        <is>
+          <t>BOQ Notification</t>
+        </is>
+      </c>
+      <c r="D31" s="31" t="inlineStr">
+        <is>
+          <t>Fix</t>
+        </is>
+      </c>
+      <c r="E31" s="29" t="inlineStr">
+        <is>
+          <t>BOQ notification send code fix</t>
+        </is>
+      </c>
+      <c r="F31" s="29" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G31" s="33" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="18" customHeight="1">
+      <c r="A32" s="26" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="26" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="C32" s="26" t="inlineStr">
+        <is>
+          <t>Vendor/Store</t>
+        </is>
+      </c>
+      <c r="D32" s="28" t="inlineStr">
+        <is>
+          <t>Fix</t>
+        </is>
+      </c>
+      <c r="E32" s="26" t="inlineStr">
+        <is>
+          <t>Vendor and store sent separately; production reject and vendor send fix</t>
+        </is>
+      </c>
+      <c r="F32" s="26" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G32" s="32" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="18" customHeight="1">
+      <c r="A33" s="29" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="29" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="C33" s="29" t="inlineStr">
+        <is>
+          <t>Notifications</t>
+        </is>
+      </c>
+      <c r="D33" s="31" t="inlineStr">
+        <is>
+          <t>Fix</t>
+        </is>
+      </c>
+      <c r="E33" s="29" t="inlineStr">
+        <is>
+          <t>Notification delivery fix</t>
+        </is>
+      </c>
+      <c r="F33" s="29" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G33" s="33" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="18" customHeight="1">
+      <c r="A34" s="26" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="26" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="C34" s="26" t="inlineStr">
+        <is>
+          <t>General Bugs</t>
+        </is>
+      </c>
+      <c r="D34" s="28" t="inlineStr">
+        <is>
+          <t>Fix</t>
+        </is>
+      </c>
+      <c r="E34" s="26" t="inlineStr">
+        <is>
+          <t>Multiple general bug fixes across backend components</t>
+        </is>
+      </c>
+      <c r="F34" s="26" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G34" s="32" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="18" customHeight="1">
+      <c r="A35" s="29" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="29" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="C35" s="29" t="inlineStr">
+        <is>
+          <t>Purchase Notification</t>
+        </is>
+      </c>
+      <c r="D35" s="31" t="inlineStr">
+        <is>
+          <t>Fix</t>
+        </is>
+      </c>
+      <c r="E35" s="29" t="inlineStr">
+        <is>
+          <t>Purchase notification fix code</t>
+        </is>
+      </c>
+      <c r="F35" s="29" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G35" s="33" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="18" customHeight="1">
+      <c r="A36" s="26" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="26" t="inlineStr">
+        <is>
+          <t>2026-02-13</t>
+        </is>
+      </c>
+      <c r="C36" s="26" t="inlineStr">
+        <is>
+          <t>TD Purchase</t>
+        </is>
+      </c>
+      <c r="D36" s="28" t="inlineStr">
+        <is>
+          <t>Fix</t>
+        </is>
+      </c>
+      <c r="E36" s="26" t="inlineStr">
+        <is>
+          <t>TD complete purchase fix</t>
+        </is>
+      </c>
+      <c r="F36" s="26" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G36" s="32" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="18" customHeight="1">
+      <c r="A37" s="29" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="29" t="inlineStr">
+        <is>
+          <t>2026-02-16</t>
+        </is>
+      </c>
+      <c r="C37" s="29" t="inlineStr">
+        <is>
+          <t>BOQ Notification</t>
+        </is>
+      </c>
+      <c r="D37" s="31" t="inlineStr">
+        <is>
+          <t>Fix</t>
+        </is>
+      </c>
+      <c r="E37" s="29" t="inlineStr">
+        <is>
+          <t>Internal revision and client revision BOQ notification fix</t>
+        </is>
+      </c>
+      <c r="F37" s="29" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G37" s="33" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="18" customHeight="1">
+      <c r="A38" s="26" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="26" t="inlineStr">
+        <is>
+          <t>2026-02-19</t>
+        </is>
+      </c>
+      <c r="C38" s="26" t="inlineStr">
+        <is>
+          <t>Duplicate Key</t>
+        </is>
+      </c>
+      <c r="D38" s="28" t="inlineStr">
+        <is>
+          <t>Fix</t>
+        </is>
+      </c>
+      <c r="E38" s="26" t="inlineStr">
+        <is>
+          <t>Duplicate drum key fix in frontend components</t>
+        </is>
+      </c>
+      <c r="F38" s="26" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G38" s="37" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="18" customHeight="1">
+      <c r="A39" s="29" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="29" t="inlineStr">
+        <is>
+          <t>2026-02-19</t>
+        </is>
+      </c>
+      <c r="C39" s="29" t="inlineStr">
+        <is>
+          <t>Email Links</t>
+        </is>
+      </c>
+      <c r="D39" s="31" t="inlineStr">
+        <is>
+          <t>Fix</t>
+        </is>
+      </c>
+      <c r="E39" s="29" t="inlineStr">
+        <is>
+          <t>Email link to open MSQ app properly</t>
+        </is>
+      </c>
+      <c r="F39" s="29" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G39" s="36" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="18" customHeight="1">
+      <c r="A40" s="26" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="26" t="inlineStr">
+        <is>
+          <t>2026-02-23</t>
+        </is>
+      </c>
+      <c r="C40" s="26" t="inlineStr">
+        <is>
+          <t>CC Mail/Vendor Email</t>
+        </is>
+      </c>
+      <c r="D40" s="28" t="inlineStr">
+        <is>
+          <t>Fix</t>
+        </is>
+      </c>
+      <c r="E40" s="26" t="inlineStr">
+        <is>
+          <t>CC mail and view vendor email fix</t>
+        </is>
+      </c>
+      <c r="F40" s="26" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G40" s="32" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="18" customHeight="1">
+      <c r="A41" s="29" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="29" t="inlineStr">
+        <is>
+          <t>2026-02-16</t>
+        </is>
+      </c>
+      <c r="C41" s="29" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+      <c r="D41" s="39" t="inlineStr">
+        <is>
+          <t>Maintenance</t>
+        </is>
+      </c>
+      <c r="E41" s="29" t="inlineStr">
+        <is>
+          <t>Removed test file from backend codebase</t>
+        </is>
+      </c>
+      <c r="F41" s="29" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G41" s="36" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="18" customHeight="1">
+      <c r="A42" s="26" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="26" t="inlineStr">
+        <is>
+          <t>2026-02-17</t>
+        </is>
+      </c>
+      <c r="C42" s="26" t="inlineStr">
+        <is>
+          <t>Offline Emails</t>
+        </is>
+      </c>
+      <c r="D42" s="38" t="inlineStr">
+        <is>
+          <t>Maintenance</t>
+        </is>
+      </c>
+      <c r="E42" s="26" t="inlineStr">
+        <is>
+          <t>Offline user email notification handling and removed backend zip file</t>
+        </is>
+      </c>
+      <c r="F42" s="26" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G42" s="37" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="18" customHeight="1">
+      <c r="A43" s="29" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="29" t="inlineStr">
+        <is>
+          <t>2026-02-18</t>
+        </is>
+      </c>
+      <c r="C43" s="29" t="inlineStr">
+        <is>
+          <t>Purchase Emails</t>
+        </is>
+      </c>
+      <c r="D43" s="39" t="inlineStr">
+        <is>
+          <t>Maintenance</t>
+        </is>
+      </c>
+      <c r="E43" s="29" t="inlineStr">
+        <is>
+          <t>Purchase email notification for offline users</t>
+        </is>
+      </c>
+      <c r="F43" s="29" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G43" s="36" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
@@ -7407,7 +9132,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9.7109375" customWidth="1" style="3" min="1" max="1"/>
@@ -7460,135 +9185,135 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>1.0.3.1</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-02-24</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>42</v>
+      </c>
+      <c r="D2" t="n">
+        <v>13</v>
+      </c>
+      <c r="E2" t="n">
+        <v>14</v>
+      </c>
+      <c r="F2" t="n">
+        <v>12</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>1.0.3.0</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-02-07</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>47</v>
+      </c>
+      <c r="D3" t="n">
+        <v>18</v>
+      </c>
+      <c r="E3" t="n">
+        <v>11</v>
+      </c>
+      <c r="F3" t="n">
+        <v>17</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Stable</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
           <t>1.0.2.1</t>
         </is>
       </c>
-      <c r="B2" s="22" t="n">
+      <c r="B4" s="22" t="n">
         <v>46040</v>
       </c>
-      <c r="C2" t="n">
+      <c r="C4" t="n">
         <v>68</v>
       </c>
-      <c r="D2" t="n">
+      <c r="D4" t="n">
         <v>25</v>
       </c>
-      <c r="E2" t="n">
+      <c r="E4" t="n">
         <v>18</v>
       </c>
-      <c r="F2" t="n">
+      <c r="F4" t="n">
         <v>25</v>
       </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Stable</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>1.0.1.5</t>
         </is>
       </c>
-      <c r="B3" s="5" t="n">
+      <c r="B5" s="5" t="n">
         <v>46022</v>
       </c>
-      <c r="C3" s="4" t="n">
+      <c r="C5" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="D3" s="4" t="n">
+      <c r="D5" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="E3" s="4" t="n">
+      <c r="E5" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="F3" s="4" t="n">
+      <c r="F5" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="G5" s="4" t="inlineStr">
         <is>
           <t>Stable</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>1.0.1.4</t>
         </is>
       </c>
-      <c r="B4" s="5" t="n">
+      <c r="B6" s="5" t="n">
         <v>46011</v>
       </c>
-      <c r="C4" s="4" t="n">
+      <c r="C6" s="4" t="n">
         <v>20</v>
       </c>
-      <c r="D4" s="4" t="n">
+      <c r="D6" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="E4" s="4" t="n">
+      <c r="E6" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="F4" s="4" t="n">
+      <c r="F6" s="4" t="n">
         <v>5</v>
-      </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>Stable</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>1.0.1.3</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>2025-12-16</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="n">
-        <v>15</v>
-      </c>
-      <c r="D5" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="E5" s="3" t="n">
-        <v>9</v>
-      </c>
-      <c r="F5" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="G5" s="3" t="inlineStr">
-        <is>
-          <t>Stable</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>1.0.1.2</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>2025-12-12</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="n">
-        <v>36</v>
-      </c>
-      <c r="D6" s="3" t="n">
-        <v>12</v>
-      </c>
-      <c r="E6" s="3" t="n">
-        <v>18</v>
-      </c>
-      <c r="F6" s="3" t="n">
-        <v>6</v>
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
@@ -7599,56 +9324,114 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>1.0.1.1</t>
+          <t>1.0.1.3</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>2025-10-12</t>
+          <t>2025-12-16</t>
         </is>
       </c>
       <c r="C7" s="3" t="n">
         <v>15</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>Legacy</t>
+          <t>Stable</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
+          <t>1.0.1.2</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>2025-12-12</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>36</v>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="F8" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>Stable</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>1.0.1.1</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>2025-10-12</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="F9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>Legacy</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
           <t>1.0.1.0</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>2025-10-01</t>
         </is>
       </c>
-      <c r="C8" s="3" t="n">
+      <c r="C10" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="D8" s="3" t="n">
+      <c r="D10" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="E8" s="3" t="n">
+      <c r="E10" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="F8" s="3" t="n">
+      <c r="F10" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="G8" s="3" t="inlineStr">
+      <c r="G10" s="3" t="inlineStr">
         <is>
           <t>Archived</t>
         </is>
@@ -7693,7 +9476,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>1.0.2.1</t>
+          <t>MSQ - MeterSquare</t>
         </is>
       </c>
     </row>
@@ -7705,7 +9488,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>1.0.2.0</t>
+          <t>1.0.3.1</t>
         </is>
       </c>
     </row>
@@ -7715,8 +9498,10 @@
           <t>Previous Version</t>
         </is>
       </c>
-      <c r="B4" s="23" t="n">
-        <v>46040</v>
+      <c r="B4" s="23" t="inlineStr">
+        <is>
+          <t>1.0.3.0</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -7727,7 +9512,7 @@
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>DevOps Team</t>
+          <t>2026-02-24</t>
         </is>
       </c>
     </row>
@@ -7739,7 +9524,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Deepika,Ramesh,Meganathan</t>
+          <t>DevOps Team</t>
         </is>
       </c>
     </row>
@@ -7751,7 +9536,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>1 (Labour workflow performance)</t>
+          <t>Production</t>
         </is>
       </c>
     </row>
@@ -7763,7 +9548,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Profit Comparison PDF, Labour Workflow, MEP Dashboard, Asset Requisition, Split API</t>
+          <t>CC Mail Fix, Vendor Email View, LPO PDF Storage, CR/TD Performance, Catalog Management</t>
         </is>
       </c>
     </row>
@@ -7775,7 +9560,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>2026-01-25</t>
+          <t>Catalog Items Management, Global Material/Labour Search, Vendor Inspection Service, LPO PDF Supabase Upload, CC Email Management, Vendor Return Flow, Online/Offline Status</t>
         </is>
       </c>
     </row>
@@ -7787,11 +9572,1716 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>2025-12-20</t>
+          <t>2026-03-07</t>
         </is>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G48"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="65" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="25" t="inlineStr">
+        <is>
+          <t>Item#</t>
+        </is>
+      </c>
+      <c r="B1" s="25" t="inlineStr">
+        <is>
+          <t>Release Date</t>
+        </is>
+      </c>
+      <c r="C1" s="25" t="inlineStr">
+        <is>
+          <t>Component</t>
+        </is>
+      </c>
+      <c r="D1" s="25" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="E1" s="25" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="F1" s="25" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="G1" s="25" t="inlineStr">
+        <is>
+          <t>Severity</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="26" t="inlineStr">
+        <is>
+          <t>2026-01-19</t>
+        </is>
+      </c>
+      <c r="C2" s="26" t="inlineStr">
+        <is>
+          <t>Labour Tracking</t>
+        </is>
+      </c>
+      <c r="D2" s="27" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E2" s="26" t="inlineStr">
+        <is>
+          <t>Added labour_role column to daily_attendance for accurate BOQ cost tracking with role-based determination logic</t>
+        </is>
+      </c>
+      <c r="F2" s="26" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G2" s="28" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="18" customHeight="1">
+      <c r="A3" s="29" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="29" t="inlineStr">
+        <is>
+          <t>2026-01-19</t>
+        </is>
+      </c>
+      <c r="C3" s="29" t="inlineStr">
+        <is>
+          <t>Labour Requisition</t>
+        </is>
+      </c>
+      <c r="D3" s="30" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E3" s="29" t="inlineStr">
+        <is>
+          <t>Enhanced labour requisition workflow with role-based security, requester role tracking, and production sending capability</t>
+        </is>
+      </c>
+      <c r="F3" s="29" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G3" s="31" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="18" customHeight="1">
+      <c r="A4" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="26" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="C4" s="26" t="inlineStr">
+        <is>
+          <t>Labour Requisition</t>
+        </is>
+      </c>
+      <c r="D4" s="27" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E4" s="26" t="inlineStr">
+        <is>
+          <t>Added TimePicker component and worker availability checks with time conflict detection for requisition assignments</t>
+        </is>
+      </c>
+      <c r="F4" s="26" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G4" s="28" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" s="29" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="29" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="C5" s="29" t="inlineStr">
+        <is>
+          <t>Labour Requisition</t>
+        </is>
+      </c>
+      <c r="D5" s="30" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E5" s="29" t="inlineStr">
+        <is>
+          <t>Added PDF download functionality for requisition assignments with improved layout and formatting</t>
+        </is>
+      </c>
+      <c r="F5" s="29" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G5" s="31" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="18" customHeight="1">
+      <c r="A6" s="26" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="26" t="inlineStr">
+        <is>
+          <t>2026-01-21</t>
+        </is>
+      </c>
+      <c r="C6" s="26" t="inlineStr">
+        <is>
+          <t>Labour PDF</t>
+        </is>
+      </c>
+      <c r="D6" s="27" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E6" s="26" t="inlineStr">
+        <is>
+          <t>Added Daily Worker Assignment Schedule PDF generator with designation, site/duty, time, and PM columns</t>
+        </is>
+      </c>
+      <c r="F6" s="26" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G6" s="32" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="18" customHeight="1">
+      <c r="A7" s="29" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="29" t="inlineStr">
+        <is>
+          <t>2026-01-22</t>
+        </is>
+      </c>
+      <c r="C7" s="29" t="inlineStr">
+        <is>
+          <t>Transport</t>
+        </is>
+      </c>
+      <c r="D7" s="30" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E7" s="29" t="inlineStr">
+        <is>
+          <t>Implemented transport flow in inventory and asset transport flow with separate routing</t>
+        </is>
+      </c>
+      <c r="F7" s="29" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G7" s="31" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="18" customHeight="1">
+      <c r="A8" s="26" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="26" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="C8" s="26" t="inlineStr">
+        <is>
+          <t>Buyer Transport</t>
+        </is>
+      </c>
+      <c r="D8" s="27" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E8" s="26" t="inlineStr">
+        <is>
+          <t>Buyer transport to site and production routing implemented</t>
+        </is>
+      </c>
+      <c r="F8" s="26" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G8" s="28" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="A9" s="29" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="29" t="inlineStr">
+        <is>
+          <t>2026-01-29</t>
+        </is>
+      </c>
+      <c r="C9" s="29" t="inlineStr">
+        <is>
+          <t>Vendor Management</t>
+        </is>
+      </c>
+      <c r="D9" s="30" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E9" s="29" t="inlineStr">
+        <is>
+          <t>Implemented vendor category management with dynamic category assignment and creation during vendor onboarding</t>
+        </is>
+      </c>
+      <c r="F9" s="29" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G9" s="31" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="A10" s="26" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="26" t="inlineStr">
+        <is>
+          <t>2026-01-30</t>
+        </is>
+      </c>
+      <c r="C10" s="26" t="inlineStr">
+        <is>
+          <t>Labour Transport</t>
+        </is>
+      </c>
+      <c r="D10" s="27" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E10" s="26" t="inlineStr">
+        <is>
+          <t>Labour transport code implementation with transport comparison in TD role and PDF fix</t>
+        </is>
+      </c>
+      <c r="F10" s="26" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G10" s="32" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="A11" s="29" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="29" t="inlineStr">
+        <is>
+          <t>2026-01-30</t>
+        </is>
+      </c>
+      <c r="C11" s="29" t="inlineStr">
+        <is>
+          <t>Admin Dashboard</t>
+        </is>
+      </c>
+      <c r="D11" s="30" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E11" s="29" t="inlineStr">
+        <is>
+          <t>Comprehensive dashboard analytics for admin with consolidated metrics in a single optimized API call</t>
+        </is>
+      </c>
+      <c r="F11" s="29" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G11" s="31" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="A12" s="26" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="26" t="inlineStr">
+        <is>
+          <t>2026-01-30</t>
+        </is>
+      </c>
+      <c r="C12" s="26" t="inlineStr">
+        <is>
+          <t>Login History</t>
+        </is>
+      </c>
+      <c r="D12" s="27" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E12" s="26" t="inlineStr">
+        <is>
+          <t>Global error handling and login history tracking for SMS OTP and email OTP authentication methods</t>
+        </is>
+      </c>
+      <c r="F12" s="26" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G12" s="28" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="18" customHeight="1">
+      <c r="A13" s="29" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="29" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="C13" s="29" t="inlineStr">
+        <is>
+          <t>BOQ Autocomplete</t>
+        </is>
+      </c>
+      <c r="D13" s="30" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E13" s="29" t="inlineStr">
+        <is>
+          <t>Global autocomplete for sub-items with duplicate prevention in master tables and new API endpoints for sub-item lookup</t>
+        </is>
+      </c>
+      <c r="F13" s="29" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G13" s="33" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="18" customHeight="1">
+      <c r="A14" s="26" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="26" t="inlineStr">
+        <is>
+          <t>2026-02-02</t>
+        </is>
+      </c>
+      <c r="C14" s="26" t="inlineStr">
+        <is>
+          <t>Estimator Dashboard</t>
+        </is>
+      </c>
+      <c r="D14" s="27" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E14" s="26" t="inlineStr">
+        <is>
+          <t>Estimator dashboard implemented with comparison view and separate item detail view</t>
+        </is>
+      </c>
+      <c r="F14" s="26" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G14" s="28" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="18" customHeight="1">
+      <c r="A15" s="29" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="29" t="inlineStr">
+        <is>
+          <t>2026-02-04</t>
+        </is>
+      </c>
+      <c r="C15" s="29" t="inlineStr">
+        <is>
+          <t>Worker PDF</t>
+        </is>
+      </c>
+      <c r="D15" s="30" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E15" s="29" t="inlineStr">
+        <is>
+          <t>Daily Worker Assignment Schedule PDF generator added for production manager role</t>
+        </is>
+      </c>
+      <c r="F15" s="29" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G15" s="33" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="18" customHeight="1">
+      <c r="A16" s="26" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="26" t="inlineStr">
+        <is>
+          <t>2026-02-05</t>
+        </is>
+      </c>
+      <c r="C16" s="26" t="inlineStr">
+        <is>
+          <t>Security Dashboard</t>
+        </is>
+      </c>
+      <c r="D16" s="27" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E16" s="26" t="inlineStr">
+        <is>
+          <t>Admin Security Dashboard with security metrics, audit logs, blocked IP management and response data masking utilities</t>
+        </is>
+      </c>
+      <c r="F16" s="26" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G16" s="28" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="18" customHeight="1">
+      <c r="A17" s="29" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="29" t="inlineStr">
+        <is>
+          <t>2026-02-05</t>
+        </is>
+      </c>
+      <c r="C17" s="29" t="inlineStr">
+        <is>
+          <t>Input Validators</t>
+        </is>
+      </c>
+      <c r="D17" s="30" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E17" s="29" t="inlineStr">
+        <is>
+          <t>Input validation utilities for sanitizing user inputs including email, phone, positive numbers and string length validation</t>
+        </is>
+      </c>
+      <c r="F17" s="29" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G17" s="31" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="18" customHeight="1">
+      <c r="A18" s="26" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="26" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="C18" s="26" t="inlineStr">
+        <is>
+          <t>Prod/Dev Security</t>
+        </is>
+      </c>
+      <c r="D18" s="27" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E18" s="26" t="inlineStr">
+        <is>
+          <t>Separate security handling for production and development environments</t>
+        </is>
+      </c>
+      <c r="F18" s="26" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G18" s="28" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="18" customHeight="1">
+      <c r="A19" s="29" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="29" t="inlineStr">
+        <is>
+          <t>2026-02-07</t>
+        </is>
+      </c>
+      <c r="C19" s="29" t="inlineStr">
+        <is>
+          <t>Asset Return</t>
+        </is>
+      </c>
+      <c r="D19" s="30" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E19" s="29" t="inlineStr">
+        <is>
+          <t>Multiple asset return type support added</t>
+        </is>
+      </c>
+      <c r="F19" s="29" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G19" s="33" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="18" customHeight="1">
+      <c r="A20" s="26" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="26" t="inlineStr">
+        <is>
+          <t>2026-01-19</t>
+        </is>
+      </c>
+      <c r="C20" s="26" t="inlineStr">
+        <is>
+          <t>Profit Comparison</t>
+        </is>
+      </c>
+      <c r="D20" s="34" t="inlineStr">
+        <is>
+          <t>Enhancement</t>
+        </is>
+      </c>
+      <c r="E20" s="26" t="inlineStr">
+        <is>
+          <t>Profit comparison status changes, margin amount fix and client amount calculation corrections</t>
+        </is>
+      </c>
+      <c r="F20" s="26" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G20" s="32" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="18" customHeight="1">
+      <c r="A21" s="29" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="29" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="C21" s="29" t="inlineStr">
+        <is>
+          <t>Labour View</t>
+        </is>
+      </c>
+      <c r="D21" s="35" t="inlineStr">
+        <is>
+          <t>Enhancement</t>
+        </is>
+      </c>
+      <c r="E21" s="29" t="inlineStr">
+        <is>
+          <t>Labour view details display time in 12-hour format in SS, PM, and PRM roles</t>
+        </is>
+      </c>
+      <c r="F21" s="29" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G21" s="36" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="18" customHeight="1">
+      <c r="A22" s="26" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="26" t="inlineStr">
+        <is>
+          <t>2026-01-21</t>
+        </is>
+      </c>
+      <c r="C22" s="26" t="inlineStr">
+        <is>
+          <t>BOQ Edit</t>
+        </is>
+      </c>
+      <c r="D22" s="34" t="inlineStr">
+        <is>
+          <t>Enhancement</t>
+        </is>
+      </c>
+      <c r="E22" s="26" t="inlineStr">
+        <is>
+          <t>Implemented BOQ edit restrictions based on PM_Approved, Items_Assigned, and Approved statuses</t>
+        </is>
+      </c>
+      <c r="F22" s="26" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G22" s="28" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="18" customHeight="1">
+      <c r="A23" s="29" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="29" t="inlineStr">
+        <is>
+          <t>2026-01-21</t>
+        </is>
+      </c>
+      <c r="C23" s="29" t="inlineStr">
+        <is>
+          <t>Labour PDF</t>
+        </is>
+      </c>
+      <c r="D23" s="35" t="inlineStr">
+        <is>
+          <t>Enhancement</t>
+        </is>
+      </c>
+      <c r="E23" s="29" t="inlineStr">
+        <is>
+          <t>Updated PDF generation for labour assignments with improved layout, new columns and formatting</t>
+        </is>
+      </c>
+      <c r="F23" s="29" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G23" s="33" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="18" customHeight="1">
+      <c r="A24" s="26" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="26" t="inlineStr">
+        <is>
+          <t>2026-01-30</t>
+        </is>
+      </c>
+      <c r="C24" s="26" t="inlineStr">
+        <is>
+          <t>Inventory Dashboard</t>
+        </is>
+      </c>
+      <c r="D24" s="34" t="inlineStr">
+        <is>
+          <t>Enhancement</t>
+        </is>
+      </c>
+      <c r="E24" s="26" t="inlineStr">
+        <is>
+          <t>Inventory dashboard includes stock health metrics and category distribution data</t>
+        </is>
+      </c>
+      <c r="F24" s="26" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G24" s="32" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="18" customHeight="1">
+      <c r="A25" s="29" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="29" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="C25" s="29" t="inlineStr">
+        <is>
+          <t>Buyer Dashboard</t>
+        </is>
+      </c>
+      <c r="D25" s="35" t="inlineStr">
+        <is>
+          <t>Enhancement</t>
+        </is>
+      </c>
+      <c r="E25" s="29" t="inlineStr">
+        <is>
+          <t>Buyer dashboard real-time purchase data synchronization with client-side pagination and updated sidebar labels</t>
+        </is>
+      </c>
+      <c r="F25" s="29" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G25" s="33" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="18" customHeight="1">
+      <c r="A26" s="26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="26" t="inlineStr">
+        <is>
+          <t>2026-02-02</t>
+        </is>
+      </c>
+      <c r="C26" s="26" t="inlineStr">
+        <is>
+          <t>Labour PDF</t>
+        </is>
+      </c>
+      <c r="D26" s="34" t="inlineStr">
+        <is>
+          <t>Enhancement</t>
+        </is>
+      </c>
+      <c r="E26" s="26" t="inlineStr">
+        <is>
+          <t>Labour transport details shown in PDF for PRM role; driver contact display fix</t>
+        </is>
+      </c>
+      <c r="F26" s="26" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G26" s="32" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="18" customHeight="1">
+      <c r="A27" s="29" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="29" t="inlineStr">
+        <is>
+          <t>2026-02-03</t>
+        </is>
+      </c>
+      <c r="C27" s="29" t="inlineStr">
+        <is>
+          <t>Asset Handling</t>
+        </is>
+      </c>
+      <c r="D27" s="35" t="inlineStr">
+        <is>
+          <t>Enhancement</t>
+        </is>
+      </c>
+      <c r="E27" s="29" t="inlineStr">
+        <is>
+          <t>Transport fee default 1 AED, individual and quantity asset handling with PDF changes</t>
+        </is>
+      </c>
+      <c r="F27" s="29" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G27" s="33" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="18" customHeight="1">
+      <c r="A28" s="26" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="26" t="inlineStr">
+        <is>
+          <t>2026-02-03</t>
+        </is>
+      </c>
+      <c r="C28" s="26" t="inlineStr">
+        <is>
+          <t>IMR/Buyer</t>
+        </is>
+      </c>
+      <c r="D28" s="34" t="inlineStr">
+        <is>
+          <t>Enhancement</t>
+        </is>
+      </c>
+      <c r="E28" s="26" t="inlineStr">
+        <is>
+          <t>Internal material request and buyer completed tab status fix with column name change for item name</t>
+        </is>
+      </c>
+      <c r="F28" s="26" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G28" s="32" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="18" customHeight="1">
+      <c r="A29" s="29" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="29" t="inlineStr">
+        <is>
+          <t>2026-02-04</t>
+        </is>
+      </c>
+      <c r="C29" s="29" t="inlineStr">
+        <is>
+          <t>BOQ Assignment</t>
+        </is>
+      </c>
+      <c r="D29" s="35" t="inlineStr">
+        <is>
+          <t>Enhancement</t>
+        </is>
+      </c>
+      <c r="E29" s="29" t="inlineStr">
+        <is>
+          <t>Enhanced get_pm_pending_boq to include checks for unassigned items and total items assigned per PM</t>
+        </is>
+      </c>
+      <c r="F29" s="29" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G29" s="33" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="18" customHeight="1">
+      <c r="A30" s="26" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="26" t="inlineStr">
+        <is>
+          <t>2026-02-04</t>
+        </is>
+      </c>
+      <c r="C30" s="26" t="inlineStr">
+        <is>
+          <t>BOQ UI</t>
+        </is>
+      </c>
+      <c r="D30" s="34" t="inlineStr">
+        <is>
+          <t>Enhancement</t>
+        </is>
+      </c>
+      <c r="E30" s="26" t="inlineStr">
+        <is>
+          <t>Estimator and PM table view change in BOQ module</t>
+        </is>
+      </c>
+      <c r="F30" s="26" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G30" s="37" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="18" customHeight="1">
+      <c r="A31" s="29" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="29" t="inlineStr">
+        <is>
+          <t>2026-02-05</t>
+        </is>
+      </c>
+      <c r="C31" s="29" t="inlineStr">
+        <is>
+          <t>N+1 Performance</t>
+        </is>
+      </c>
+      <c r="D31" s="35" t="inlineStr">
+        <is>
+          <t>Enhancement</t>
+        </is>
+      </c>
+      <c r="E31" s="29" t="inlineStr">
+        <is>
+          <t>Eager loading implemented for AssetDeliveryNote, AssetReturnDeliveryNote, InventoryTransaction, and MaterialDeliveryNote queries</t>
+        </is>
+      </c>
+      <c r="F31" s="29" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G31" s="31" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="18" customHeight="1">
+      <c r="A32" s="26" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="26" t="inlineStr">
+        <is>
+          <t>2026-02-05</t>
+        </is>
+      </c>
+      <c r="C32" s="26" t="inlineStr">
+        <is>
+          <t>Labour Edit</t>
+        </is>
+      </c>
+      <c r="D32" s="34" t="inlineStr">
+        <is>
+          <t>Enhancement</t>
+        </is>
+      </c>
+      <c r="E32" s="26" t="inlineStr">
+        <is>
+          <t>Edit functionality for labour requisitions added in RequisitionApprovals with pre-fill support and time validation</t>
+        </is>
+      </c>
+      <c r="F32" s="26" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G32" s="32" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="18" customHeight="1">
+      <c r="A33" s="29" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="29" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="C33" s="29" t="inlineStr">
+        <is>
+          <t>Transport Fee</t>
+        </is>
+      </c>
+      <c r="D33" s="35" t="inlineStr">
+        <is>
+          <t>Enhancement</t>
+        </is>
+      </c>
+      <c r="E33" s="29" t="inlineStr">
+        <is>
+          <t>Transport fee and delivery notes displayed in PRM stock page</t>
+        </is>
+      </c>
+      <c r="F33" s="29" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G33" s="33" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="18" customHeight="1">
+      <c r="A34" s="26" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="26" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="C34" s="26" t="inlineStr">
+        <is>
+          <t>Asset Routes</t>
+        </is>
+      </c>
+      <c r="D34" s="34" t="inlineStr">
+        <is>
+          <t>Enhancement</t>
+        </is>
+      </c>
+      <c r="E34" s="26" t="inlineStr">
+        <is>
+          <t>Proper routing set for asset management and terms &amp; conditions</t>
+        </is>
+      </c>
+      <c r="F34" s="26" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G34" s="37" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="18" customHeight="1">
+      <c r="A35" s="29" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="29" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="C35" s="29" t="inlineStr">
+        <is>
+          <t>Purchase Update</t>
+        </is>
+      </c>
+      <c r="D35" s="35" t="inlineStr">
+        <is>
+          <t>Enhancement</t>
+        </is>
+      </c>
+      <c r="E35" s="29" t="inlineStr">
+        <is>
+          <t>Purchase flow update with vendor create and PO completed flow</t>
+        </is>
+      </c>
+      <c r="F35" s="29" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G35" s="33" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="18" customHeight="1">
+      <c r="A36" s="26" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="26" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="C36" s="26" t="inlineStr">
+        <is>
+          <t>BOQ Fixes</t>
+        </is>
+      </c>
+      <c r="D36" s="34" t="inlineStr">
+        <is>
+          <t>Enhancement</t>
+        </is>
+      </c>
+      <c r="E36" s="26" t="inlineStr">
+        <is>
+          <t>BOQ create and view issue fixes</t>
+        </is>
+      </c>
+      <c r="F36" s="26" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G36" s="32" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="18" customHeight="1">
+      <c r="A37" s="29" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="29" t="inlineStr">
+        <is>
+          <t>2026-01-21</t>
+        </is>
+      </c>
+      <c r="C37" s="29" t="inlineStr">
+        <is>
+          <t>Estimator</t>
+        </is>
+      </c>
+      <c r="D37" s="31" t="inlineStr">
+        <is>
+          <t>Fix</t>
+        </is>
+      </c>
+      <c r="E37" s="29" t="inlineStr">
+        <is>
+          <t>Estimator tab count mismatch fix</t>
+        </is>
+      </c>
+      <c r="F37" s="29" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G37" s="33" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="18" customHeight="1">
+      <c r="A38" s="26" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="26" t="inlineStr">
+        <is>
+          <t>2026-01-21</t>
+        </is>
+      </c>
+      <c r="C38" s="26" t="inlineStr">
+        <is>
+          <t>MRP Stock</t>
+        </is>
+      </c>
+      <c r="D38" s="28" t="inlineStr">
+        <is>
+          <t>Fix</t>
+        </is>
+      </c>
+      <c r="E38" s="26" t="inlineStr">
+        <is>
+          <t>Transaction in MRP role stock-in page fixed</t>
+        </is>
+      </c>
+      <c r="F38" s="26" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G38" s="32" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="18" customHeight="1">
+      <c r="A39" s="29" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="29" t="inlineStr">
+        <is>
+          <t>2026-02-02</t>
+        </is>
+      </c>
+      <c r="C39" s="29" t="inlineStr">
+        <is>
+          <t>Delivery Note</t>
+        </is>
+      </c>
+      <c r="D39" s="31" t="inlineStr">
+        <is>
+          <t>Fix</t>
+        </is>
+      </c>
+      <c r="E39" s="29" t="inlineStr">
+        <is>
+          <t>Updated delivery note download API endpoint to include inventory path</t>
+        </is>
+      </c>
+      <c r="F39" s="29" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G39" s="33" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="18" customHeight="1">
+      <c r="A40" s="26" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="26" t="inlineStr">
+        <is>
+          <t>2026-02-02</t>
+        </is>
+      </c>
+      <c r="C40" s="26" t="inlineStr">
+        <is>
+          <t>Budget</t>
+        </is>
+      </c>
+      <c r="D40" s="28" t="inlineStr">
+        <is>
+          <t>Fix</t>
+        </is>
+      </c>
+      <c r="E40" s="26" t="inlineStr">
+        <is>
+          <t>Comparison UI and mismatch budget fix; removed My Request section from buyer</t>
+        </is>
+      </c>
+      <c r="F40" s="26" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G40" s="32" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="18" customHeight="1">
+      <c r="A41" s="29" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="29" t="inlineStr">
+        <is>
+          <t>2026-02-04</t>
+        </is>
+      </c>
+      <c r="C41" s="29" t="inlineStr">
+        <is>
+          <t>Projects</t>
+        </is>
+      </c>
+      <c r="D41" s="31" t="inlineStr">
+        <is>
+          <t>Fix</t>
+        </is>
+      </c>
+      <c r="E41" s="29" t="inlineStr">
+        <is>
+          <t>Removed priority handling from MyProjects, ProjectApprovals, and SiteEngineer components</t>
+        </is>
+      </c>
+      <c r="F41" s="29" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G41" s="36" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="18" customHeight="1">
+      <c r="A42" s="26" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="26" t="inlineStr">
+        <is>
+          <t>2026-02-04</t>
+        </is>
+      </c>
+      <c r="C42" s="26" t="inlineStr">
+        <is>
+          <t>DB Session</t>
+        </is>
+      </c>
+      <c r="D42" s="28" t="inlineStr">
+        <is>
+          <t>Fix</t>
+        </is>
+      </c>
+      <c r="E42" s="26" t="inlineStr">
+        <is>
+          <t>Database session cleanup and error handling after each request implemented</t>
+        </is>
+      </c>
+      <c r="F42" s="26" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G42" s="32" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="18" customHeight="1">
+      <c r="A43" s="29" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="29" t="inlineStr">
+        <is>
+          <t>2026-02-05</t>
+        </is>
+      </c>
+      <c r="C43" s="29" t="inlineStr">
+        <is>
+          <t>Labour Time</t>
+        </is>
+      </c>
+      <c r="D43" s="31" t="inlineStr">
+        <is>
+          <t>Fix</t>
+        </is>
+      </c>
+      <c r="E43" s="29" t="inlineStr">
+        <is>
+          <t>Labour time update and time validation (end time after start time) in requisition forms</t>
+        </is>
+      </c>
+      <c r="F43" s="29" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G43" s="33" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="18" customHeight="1">
+      <c r="A44" s="26" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="26" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="C44" s="26" t="inlineStr">
+        <is>
+          <t>Stock Check</t>
+        </is>
+      </c>
+      <c r="D44" s="28" t="inlineStr">
+        <is>
+          <t>Fix</t>
+        </is>
+      </c>
+      <c r="E44" s="26" t="inlineStr">
+        <is>
+          <t>Stock check and availability validation fix</t>
+        </is>
+      </c>
+      <c r="F44" s="26" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G44" s="32" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="18" customHeight="1">
+      <c r="A45" s="29" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="29" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="C45" s="29" t="inlineStr">
+        <is>
+          <t>Debug Print</t>
+        </is>
+      </c>
+      <c r="D45" s="31" t="inlineStr">
+        <is>
+          <t>Fix</t>
+        </is>
+      </c>
+      <c r="E45" s="29" t="inlineStr">
+        <is>
+          <t>Removed debug print statement from codebase</t>
+        </is>
+      </c>
+      <c r="F45" s="29" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G45" s="36" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="18" customHeight="1">
+      <c r="A46" s="26" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="26" t="inlineStr">
+        <is>
+          <t>2026-02-07</t>
+        </is>
+      </c>
+      <c r="C46" s="26" t="inlineStr">
+        <is>
+          <t>Material Bugs</t>
+        </is>
+      </c>
+      <c r="D46" s="28" t="inlineStr">
+        <is>
+          <t>Fix</t>
+        </is>
+      </c>
+      <c r="E46" s="26" t="inlineStr">
+        <is>
+          <t>Material display and processing bugs fixed</t>
+        </is>
+      </c>
+      <c r="F46" s="26" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G46" s="32" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="18" customHeight="1">
+      <c r="A47" s="29" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="29" t="inlineStr">
+        <is>
+          <t>2026-02-07</t>
+        </is>
+      </c>
+      <c r="C47" s="29" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="D47" s="31" t="inlineStr">
+        <is>
+          <t>Fix</t>
+        </is>
+      </c>
+      <c r="E47" s="29" t="inlineStr">
+        <is>
+          <t>General bug fixes across multiple components</t>
+        </is>
+      </c>
+      <c r="F47" s="29" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G47" s="36" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="18" customHeight="1">
+      <c r="A48" s="26" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="26" t="inlineStr">
+        <is>
+          <t>2026-01-19</t>
+        </is>
+      </c>
+      <c r="C48" s="26" t="inlineStr">
+        <is>
+          <t>Codebase</t>
+        </is>
+      </c>
+      <c r="D48" s="38" t="inlineStr">
+        <is>
+          <t>Maintenance</t>
+        </is>
+      </c>
+      <c r="E48" s="26" t="inlineStr">
+        <is>
+          <t>Removed unused migration file and test files from backend</t>
+        </is>
+      </c>
+      <c r="F48" s="26" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G48" s="37" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
version update in excel file
</commit_message>
<xml_diff>
--- a/MSQ App Version History.xlsx
+++ b/MSQ App Version History.xlsx
@@ -743,7 +743,7 @@
       </c>
       <c r="F2" s="24" t="inlineStr">
         <is>
-          <t>Latest - 42 features/fixes</t>
+          <t>Latest - 55 features/fixes</t>
         </is>
       </c>
     </row>
@@ -1008,7 +1008,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G43"/>
+  <dimension ref="A1:G56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2524,6 +2524,461 @@
       <c r="G43" s="36" t="inlineStr">
         <is>
           <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>2026-02-24</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Buyer UI</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Enhancement</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Buyer item display improved - show code changes for better item visibility in buyer role</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>2026-02-24</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Performance</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Enhancement</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>N+1 query optimization in buyer endpoints - batch pre-fetch related records to reduce DB calls</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>2026-02-24</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Version</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Maintenance</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Version reference (vr) update for release tracking</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>2026-02-25</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Production Manager</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Enhancement</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Production manager notification system updated for better delivery and tracking</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>2026-02-25</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Frontend UI</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Animated particles background UI component added for visual enhancement on landing screens</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>2026-02-25</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Performance</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Enhancement</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Batch pre-fetching implemented for buyer PO child endpoints to fully eliminate N+1 queries</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>2026-02-26</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Procurement</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Fix</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Procurement notification page navigation fix - correct redirect after notification action</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>2026-02-27</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Site Assets</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Enhancement</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>SiteAssets Cancel button hidden until Cancelled tab implemented; VAT percent input placeholder removed</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>2026-02-27</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Notifications</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Enhancement</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Notification polling service improved with desktop notification support and unread handling via realtimeNotificationHub</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>2026-02-27</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>TD Search</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Fix</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>TD (Technical Director) search functionality fix</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>2026-02-27</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>PRM Role</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Fix</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Worker code edit and add functionality fix in PRM (Production Manager) role</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>2026-02-27</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Admin Dashboard</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Fix</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Admin dashboard display and functionality fix</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>2026-02-28</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>TD Role</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Report page implemented in TD (Technical Director) role for project reporting</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>

</xml_diff>